<commit_message>
Journal rapport de raphael
</commit_message>
<xml_diff>
--- a/planning/Journal_mariet_raphael.xlsx
+++ b/planning/Journal_mariet_raphael.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raphael.mariet\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raphael.mariet\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{44327D69-E427-4C23-B574-4330A791A3BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AFAECF7-ECB9-4601-B669-976E58467E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{9E606028-D228-4CF5-9D9A-B028276625EA}"/>
+    <workbookView xWindow="6150" yWindow="2865" windowWidth="21600" windowHeight="11295" xr2:uid="{9E606028-D228-4CF5-9D9A-B028276625EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -38,62 +38,63 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
   <si>
-    <t>Heure de fin</t>
-  </si>
-  <si>
-    <t>9h25</t>
-  </si>
-  <si>
-    <t>1h05</t>
-  </si>
-  <si>
-    <t>11h20</t>
-  </si>
-  <si>
-    <t>1h55</t>
-  </si>
-  <si>
-    <t>Etape Mini-Projet</t>
-  </si>
-  <si>
-    <t>Séance réalisé</t>
-  </si>
-  <si>
-    <t>n°3</t>
-  </si>
-  <si>
-    <t>Création de la Fonction filtre pseudo</t>
-  </si>
-  <si>
-    <t>Création de la Fonction Send-Error</t>
-  </si>
-  <si>
-    <t>Durée</t>
-  </si>
-  <si>
-    <t>Implémentation des 2 fonctions dans le projet</t>
-  </si>
-  <si>
-    <t>30min</t>
-  </si>
-  <si>
-    <t>11h50</t>
-  </si>
-  <si>
-    <t>Diagramme de séquence</t>
-  </si>
-  <si>
-    <t>10min</t>
-  </si>
-  <si>
-    <t>12h05</t>
+    <t>Jour</t>
+  </si>
+  <si>
+    <t>Nombre total d’heures travaillées</t>
+  </si>
+  <si>
+    <t>Séances</t>
+  </si>
+  <si>
+    <t>Détails des tâches effectuées</t>
+  </si>
+  <si>
+    <t>4H</t>
+  </si>
+  <si>
+    <t>Séances 1</t>
+  </si>
+  <si>
+    <t>1H</t>
+  </si>
+  <si>
+    <t>Séances 2</t>
+  </si>
+  <si>
+    <t>Séances 3</t>
+  </si>
+  <si>
+    <t>Séances 4</t>
+  </si>
+  <si>
+    <t>Séances 5</t>
+  </si>
+  <si>
+    <t>Journal d’activité – Projet SquidTchat – Raphaël MARIET</t>
+  </si>
+  <si>
+    <t>Rédaction du cahier des charges, réalisation des diagrammes de cas d'utilisation, initialisation des filtres des pseudos.</t>
+  </si>
+  <si>
+    <t>Développement et correction du cahier des charges.</t>
+  </si>
+  <si>
+    <t>Réalisation du diagramme de séquence, finalisation de la fonction filtre des pseudos et création de la fonction send error.</t>
+  </si>
+  <si>
+    <t>Création du filtre de message, Mise en oeuvre des premiers cahiers de recette, 
+mise à jour de l'html avec wilstan pour l'affichage du titre</t>
+  </si>
+  <si>
+    <t>Finalisation des filtres pseudos, présentation finale du projet, finalisations des derniers cahiers de recette</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,13 +102,32 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -137,28 +157,43 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -494,165 +529,344 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{321867BA-58C3-4039-9B9D-E0C84A3541D7}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" customWidth="1"/>
-    <col min="2" max="12" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="22.5703125" customWidth="1"/>
+    <col min="2" max="2" width="35.5703125" customWidth="1"/>
+    <col min="3" max="4" width="17.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="7"/>
+    </row>
+    <row r="2" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="7"/>
+      <c r="B2" s="7"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="7"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+    </row>
+    <row r="3" spans="1:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4"/>
+    </row>
+    <row r="4" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="6" t="s">
+      <c r="D4" s="5"/>
+      <c r="E4" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+    </row>
+    <row r="5" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>46098</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="5"/>
+    </row>
+    <row r="6" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>46104</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+      <c r="H6" s="6"/>
+      <c r="I6" s="6"/>
+    </row>
+    <row r="7" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>46115</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="5"/>
+      <c r="E7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="6"/>
+      <c r="G7" s="6"/>
+      <c r="H7" s="6"/>
+      <c r="I7" s="6"/>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>46139</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
-    </row>
-    <row r="2" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="1"/>
-      <c r="I2" s="1"/>
-      <c r="J2" s="1"/>
-      <c r="K2" s="1"/>
-    </row>
-    <row r="3" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
-      <c r="K3" s="1"/>
-    </row>
-    <row r="4" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="1"/>
-      <c r="I4" s="1"/>
-      <c r="J4" s="1"/>
-      <c r="K4" s="1"/>
-    </row>
-    <row r="5" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="D8" s="5"/>
+      <c r="E8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="1"/>
-    </row>
-    <row r="6" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="6"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="4"/>
-      <c r="F6" s="4"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1"/>
-      <c r="J6" s="1"/>
-      <c r="K6" s="1"/>
-    </row>
-    <row r="7" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="6"/>
-      <c r="B7" s="6"/>
-      <c r="C7" s="6"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="5"/>
-      <c r="F7" s="5"/>
-      <c r="G7" s="3"/>
-    </row>
-    <row r="8" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="6"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="5"/>
-      <c r="F8" s="5"/>
-      <c r="G8" s="3"/>
-    </row>
-    <row r="9" spans="1:11" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="6"/>
-      <c r="B9" s="6"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="6"/>
+      <c r="H8" s="6"/>
+      <c r="I8" s="6"/>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="10"/>
+      <c r="C9" s="10"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="10"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="10"/>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="10"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="10"/>
+      <c r="D10" s="10"/>
+      <c r="E10" s="10"/>
+      <c r="F10" s="10"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="10"/>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="10"/>
+      <c r="B11" s="10"/>
+      <c r="C11" s="10"/>
+      <c r="D11" s="10"/>
+      <c r="E11" s="10"/>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="10"/>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="10"/>
+      <c r="B12" s="10"/>
+      <c r="C12" s="10"/>
+      <c r="D12" s="10"/>
+      <c r="E12" s="10"/>
+      <c r="F12" s="10"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="10"/>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+      <c r="I13" s="12"/>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="10"/>
+      <c r="C15" s="10"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="10"/>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="10"/>
+      <c r="B16" s="10"/>
+      <c r="C16" s="10"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="10"/>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="10"/>
+      <c r="C17" s="10"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="10"/>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="10"/>
+      <c r="B18" s="10"/>
+      <c r="C18" s="10"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="10"/>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="10"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="10"/>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="10"/>
+      <c r="B20" s="10"/>
+      <c r="C20" s="10"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="10"/>
     </row>
   </sheetData>
+  <mergeCells count="34">
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="E8:I8"/>
+    <mergeCell ref="C19:D20"/>
+    <mergeCell ref="A19:A20"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="E19:I20"/>
+    <mergeCell ref="E9:I10"/>
+    <mergeCell ref="E11:I12"/>
+    <mergeCell ref="C9:D10"/>
+    <mergeCell ref="C11:D12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C15:D16"/>
+    <mergeCell ref="C17:D18"/>
+    <mergeCell ref="A13:I14"/>
+    <mergeCell ref="E15:I16"/>
+    <mergeCell ref="E17:I18"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E7:I7"/>
+    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="E4:I4"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E3DBFDA92D80EA48A7EED411DA26BC07" ma:contentTypeVersion="9" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="8d7da3b0ce409c83d2d88bc67c89ad87">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="61a5eff35266d42fcf39f049a9a05b65" ns3:_="">
     <xsd:import namespace="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
@@ -828,24 +1042,31 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8215EF4-8B6C-4F4D-BD74-6E67CB8A9565}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E005873-B806-4D16-8477-98C226AA4228}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47E4EB07-CDF5-48C7-A776-2D8C4B65E6D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -861,28 +1082,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E005873-B806-4D16-8477-98C226AA4228}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8215EF4-8B6C-4F4D-BD74-6E67CB8A9565}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Maj du rapport raphael
</commit_message>
<xml_diff>
--- a/planning/Journal_mariet_raphael.xlsx
+++ b/planning/Journal_mariet_raphael.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\raphael.mariet\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3AFAECF7-ECB9-4601-B669-976E58467E94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8601844-C7FB-4AE7-B1CE-9D0B17F4FC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6150" yWindow="2865" windowWidth="21600" windowHeight="11295" xr2:uid="{9E606028-D228-4CF5-9D9A-B028276625EA}"/>
+    <workbookView xWindow="1500" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{9E606028-D228-4CF5-9D9A-B028276625EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -157,15 +157,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -177,22 +174,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -538,28 +535,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11"/>
+      <c r="D1" s="11"/>
+      <c r="E1" s="11"/>
+      <c r="F1" s="11"/>
+      <c r="G1" s="11"/>
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
     </row>
     <row r="2" spans="1:9" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
     </row>
     <row r="3" spans="1:9" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
@@ -568,17 +565,17 @@
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4" t="s">
+      <c r="D3" s="10"/>
+      <c r="E3" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
+      <c r="F3" s="10"/>
+      <c r="G3" s="10"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="10"/>
     </row>
     <row r="4" spans="1:9" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -587,17 +584,17 @@
       <c r="B4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="6" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="6"/>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
-      <c r="I4" s="6"/>
+      <c r="F4" s="5"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
+      <c r="I4" s="5"/>
     </row>
     <row r="5" spans="1:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -606,17 +603,17 @@
       <c r="B5" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5" t="s">
+      <c r="D5" s="4"/>
+      <c r="E5" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
-      <c r="I5" s="5"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
+      <c r="I5" s="4"/>
     </row>
     <row r="6" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
@@ -625,17 +622,17 @@
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="5"/>
-      <c r="E6" s="6" t="s">
+      <c r="D6" s="4"/>
+      <c r="E6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="F6" s="6"/>
-      <c r="G6" s="6"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="F6" s="5"/>
+      <c r="G6" s="5"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
     </row>
     <row r="7" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
@@ -644,171 +641,189 @@
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="5"/>
-      <c r="E7" s="6" t="s">
+      <c r="D7" s="4"/>
+      <c r="E7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="5"/>
+      <c r="I7" s="5"/>
+    </row>
+    <row r="8" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>46139</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="5"/>
-      <c r="E8" s="6" t="s">
+      <c r="D8" s="4"/>
+      <c r="E8" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
+      <c r="F8" s="5"/>
+      <c r="G8" s="5"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="5"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" s="10"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="6"/>
+      <c r="H9" s="6"/>
+      <c r="I9" s="6"/>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" s="10"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="6"/>
+      <c r="H10" s="6"/>
+      <c r="I10" s="6"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="6"/>
+      <c r="H11" s="6"/>
+      <c r="I11" s="6"/>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="6"/>
+      <c r="H12" s="6"/>
+      <c r="I12" s="6"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A15" s="9"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="6"/>
+      <c r="H15" s="6"/>
+      <c r="I15" s="6"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="6"/>
+      <c r="H16" s="6"/>
+      <c r="I16" s="6"/>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A17" s="9"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="6"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
     </row>
     <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="9"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="6"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="10"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="6"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="34">
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="E7:I7"/>
+    <mergeCell ref="A1:I2"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="A13:I14"/>
+    <mergeCell ref="E15:I16"/>
+    <mergeCell ref="E17:I18"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="A17:A18"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="E8:I8"/>
     <mergeCell ref="C19:D20"/>
@@ -825,24 +840,6 @@
     <mergeCell ref="B9:B10"/>
     <mergeCell ref="C15:D16"/>
     <mergeCell ref="C17:D18"/>
-    <mergeCell ref="A13:I14"/>
-    <mergeCell ref="E15:I16"/>
-    <mergeCell ref="E17:I18"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="A17:A18"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="E7:I7"/>
-    <mergeCell ref="A1:I2"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="E4:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
@@ -850,23 +847,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E3DBFDA92D80EA48A7EED411DA26BC07" ma:contentTypeVersion="9" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="8d7da3b0ce409c83d2d88bc67c89ad87">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="61a5eff35266d42fcf39f049a9a05b65" ns3:_="">
     <xsd:import namespace="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
@@ -1042,31 +1022,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8215EF4-8B6C-4F4D-BD74-6E67CB8A9565}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E005873-B806-4D16-8477-98C226AA4228}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{47E4EB07-CDF5-48C7-A776-2D8C4B65E6D4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1082,4 +1055,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8E005873-B806-4D16-8477-98C226AA4228}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B8215EF4-8B6C-4F4D-BD74-6E67CB8A9565}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="25b9d25b-f3e3-4424-a4f0-1b70bb014b4c"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>